<commit_message>
create base allocator class
</commit_message>
<xml_diff>
--- a/results/greedy/UAVs10_GRID13/revenue/UAVs10_GRID13_Greedy.xlsx
+++ b/results/greedy/UAVs10_GRID13/revenue/UAVs10_GRID13_Greedy.xlsx
@@ -582,7 +582,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02230304200202227</v>
+        <v>0.0228276249836199</v>
       </c>
       <c r="C2" t="n">
         <v>16.76998776594836</v>
@@ -696,7 +696,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.01524516701465473</v>
+        <v>0.01510970795061439</v>
       </c>
       <c r="C2" t="n">
         <v>16.0492781967595</v>
@@ -810,7 +810,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02101450000191107</v>
+        <v>0.02123937499709427</v>
       </c>
       <c r="C2" t="n">
         <v>18.98038184304531</v>
@@ -924,7 +924,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02169699996011332</v>
+        <v>0.02133658301318064</v>
       </c>
       <c r="C2" t="n">
         <v>15.89495908648763</v>
@@ -1038,7 +1038,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02075562498066574</v>
+        <v>0.01915641705272719</v>
       </c>
       <c r="C2" t="n">
         <v>17.92737718894672</v>
@@ -1152,7 +1152,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.01765820803120732</v>
+        <v>0.01747616700595245</v>
       </c>
       <c r="C2" t="n">
         <v>24.03421134451127</v>
@@ -1266,7 +1266,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02532129199244082</v>
+        <v>0.02523191599175334</v>
       </c>
       <c r="C2" t="n">
         <v>15.65089684964522</v>
@@ -1380,7 +1380,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02485987503314391</v>
+        <v>0.02416158397682011</v>
       </c>
       <c r="C2" t="n">
         <v>18.62783117024307</v>
@@ -1494,7 +1494,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02388074999907985</v>
+        <v>0.02344716695370153</v>
       </c>
       <c r="C2" t="n">
         <v>17.40462171047929</v>
@@ -1608,7 +1608,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02512662502704188</v>
+        <v>0.02472437504911795</v>
       </c>
       <c r="C2" t="n">
         <v>21.82867308882576</v>
@@ -1722,7 +1722,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.01756608398864046</v>
+        <v>0.01833412499399856</v>
       </c>
       <c r="C2" t="n">
         <v>19.55337090416027</v>
@@ -1836,7 +1836,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02076962502906099</v>
+        <v>0.02074308396549895</v>
       </c>
       <c r="C2" t="n">
         <v>17.14559081924716</v>
@@ -1950,7 +1950,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.0242477499996312</v>
+        <v>0.02404291700804606</v>
       </c>
       <c r="C2" t="n">
         <v>22.56190618819002</v>
@@ -2064,7 +2064,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02482474996941164</v>
+        <v>0.02499566599726677</v>
       </c>
       <c r="C2" t="n">
         <v>20.32014892302262</v>
@@ -2178,7 +2178,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02276379195973277</v>
+        <v>0.02406916697509587</v>
       </c>
       <c r="C2" t="n">
         <v>16.05463846747012</v>
@@ -2292,7 +2292,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02471716701984406</v>
+        <v>0.02521237498149276</v>
       </c>
       <c r="C2" t="n">
         <v>22.87030402180811</v>
@@ -2406,7 +2406,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02419145795283839</v>
+        <v>0.02323833300033584</v>
       </c>
       <c r="C2" t="n">
         <v>19.8048688092705</v>
@@ -2520,7 +2520,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02319466701010242</v>
+        <v>0.02334737504133955</v>
       </c>
       <c r="C2" t="n">
         <v>15.13985900559922</v>
@@ -2634,7 +2634,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02121074998285621</v>
+        <v>0.02080679195933044</v>
       </c>
       <c r="C2" t="n">
         <v>17.0796708864229</v>
@@ -2748,7 +2748,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.0219158330000937</v>
+        <v>0.02236491697840393</v>
       </c>
       <c r="C2" t="n">
         <v>19.08806867117367</v>
@@ -2862,7 +2862,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02151958300964907</v>
+        <v>0.02181083400500938</v>
       </c>
       <c r="C2" t="n">
         <v>17.59812025522887</v>
@@ -2976,7 +2976,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02316970902029425</v>
+        <v>0.02480416698381305</v>
       </c>
       <c r="C2" t="n">
         <v>22.90102452797837</v>
@@ -3090,7 +3090,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.01877462497213855</v>
+        <v>0.02122879197122529</v>
       </c>
       <c r="C2" t="n">
         <v>18.34141271881758</v>
@@ -3204,7 +3204,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.01930408301996067</v>
+        <v>0.01913475000765175</v>
       </c>
       <c r="C2" t="n">
         <v>20.53784612898966</v>
@@ -3318,7 +3318,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02280908398097381</v>
+        <v>0.02317954105092213</v>
       </c>
       <c r="C2" t="n">
         <v>19.44152347277755</v>
@@ -3432,7 +3432,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02254720800556242</v>
+        <v>0.02237441600300372</v>
       </c>
       <c r="C2" t="n">
         <v>15.14196692208723</v>
@@ -3546,7 +3546,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.01857804198516533</v>
+        <v>0.01883974997326732</v>
       </c>
       <c r="C2" t="n">
         <v>13.71798871009618</v>
@@ -3660,7 +3660,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.01582733303075656</v>
+        <v>0.01579791697440669</v>
       </c>
       <c r="C2" t="n">
         <v>16.88235167036955</v>
@@ -3774,7 +3774,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02214862499386072</v>
+        <v>0.02116016601212323</v>
       </c>
       <c r="C2" t="n">
         <v>17.80508116359996</v>
@@ -3888,7 +3888,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.01897899998584762</v>
+        <v>0.01875008299248293</v>
       </c>
       <c r="C2" t="n">
         <v>13.90745992226739</v>
@@ -4002,7 +4002,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02079366601537913</v>
+        <v>0.02011566696455702</v>
       </c>
       <c r="C2" t="n">
         <v>20.76446807284532</v>
@@ -4116,7 +4116,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02191616699565202</v>
+        <v>0.02255208301357925</v>
       </c>
       <c r="C2" t="n">
         <v>15.79919247978209</v>
@@ -4230,7 +4230,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02141124999616295</v>
+        <v>0.02123150002444163</v>
       </c>
       <c r="C2" t="n">
         <v>21.9332762481501</v>
@@ -4344,7 +4344,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02213858300819993</v>
+        <v>0.02282441698480397</v>
       </c>
       <c r="C2" t="n">
         <v>18.86980496379388</v>
@@ -4458,7 +4458,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02097908401628956</v>
+        <v>0.02055049996124581</v>
       </c>
       <c r="C2" t="n">
         <v>14.53929702107344</v>
@@ -4572,7 +4572,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.0209497920004651</v>
+        <v>0.02180812502047047</v>
       </c>
       <c r="C2" t="n">
         <v>17.99358070168426</v>
@@ -4686,7 +4686,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02028662501834333</v>
+        <v>0.02069395803846419</v>
       </c>
       <c r="C2" t="n">
         <v>19.87851972194529</v>
@@ -4800,7 +4800,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02301929204259068</v>
+        <v>0.02318829199066386</v>
       </c>
       <c r="C2" t="n">
         <v>22.07078986231716</v>
@@ -4914,7 +4914,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.01871475001098588</v>
+        <v>0.01813716697506607</v>
       </c>
       <c r="C2" t="n">
         <v>13.68699789963908</v>
@@ -5028,7 +5028,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.01889795798342675</v>
+        <v>0.0192385419504717</v>
       </c>
       <c r="C2" t="n">
         <v>14.09813465732448</v>
@@ -5142,7 +5142,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02177158300764859</v>
+        <v>0.02219904196681455</v>
       </c>
       <c r="C2" t="n">
         <v>16.24276270949859</v>
@@ -5256,7 +5256,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02719833300216123</v>
+        <v>0.02697758300928399</v>
       </c>
       <c r="C2" t="n">
         <v>22.48223127691992</v>
@@ -5370,7 +5370,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02228191698668525</v>
+        <v>0.02160179201746359</v>
       </c>
       <c r="C2" t="n">
         <v>19.03741151629958</v>
@@ -5484,7 +5484,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02361233299598098</v>
+        <v>0.0231659589917399</v>
       </c>
       <c r="C2" t="n">
         <v>18.77205748518454</v>
@@ -5598,7 +5598,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02119599998695776</v>
+        <v>0.02043595799477771</v>
       </c>
       <c r="C2" t="n">
         <v>16.40841271252996</v>
@@ -5712,7 +5712,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02298770798370242</v>
+        <v>0.02237437502481043</v>
       </c>
       <c r="C2" t="n">
         <v>16.10627050452097</v>
@@ -5826,7 +5826,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02658325002994388</v>
+        <v>0.02644891705131158</v>
       </c>
       <c r="C2" t="n">
         <v>24.84666489475304</v>
@@ -5940,7 +5940,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.0229863750282675</v>
+        <v>0.02201483299722895</v>
       </c>
       <c r="C2" t="n">
         <v>20.75614653023874</v>
@@ -6054,7 +6054,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02574675000505522</v>
+        <v>0.02470312500372529</v>
       </c>
       <c r="C2" t="n">
         <v>20.9551086688087</v>
@@ -6168,7 +6168,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.01962199999252334</v>
+        <v>0.01975787500850856</v>
       </c>
       <c r="C2" t="n">
         <v>17.48585309601928</v>
@@ -6282,7 +6282,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02411025000037625</v>
+        <v>0.0231932089664042</v>
       </c>
       <c r="C2" t="n">
         <v>17.11346165273365</v>
@@ -6396,7 +6396,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02132966701174155</v>
+        <v>0.02045887499116361</v>
       </c>
       <c r="C2" t="n">
         <v>19.64311531557314</v>
@@ -6510,7 +6510,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.01805799995781854</v>
+        <v>0.01730191597016528</v>
       </c>
       <c r="C2" t="n">
         <v>21.4405152123048</v>
@@ -6624,7 +6624,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02581687504425645</v>
+        <v>0.0250022909604013</v>
       </c>
       <c r="C2" t="n">
         <v>27.23987562532511</v>
@@ -6738,7 +6738,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02035025000805035</v>
+        <v>0.01942799997050315</v>
       </c>
       <c r="C2" t="n">
         <v>15.76247057293731</v>
@@ -6852,7 +6852,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02313479199074209</v>
+        <v>0.02266104199225083</v>
       </c>
       <c r="C2" t="n">
         <v>15.38083796261023</v>
@@ -6966,7 +6966,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02394983300473541</v>
+        <v>0.02334541600430384</v>
       </c>
       <c r="C2" t="n">
         <v>28.46291318848075</v>
@@ -7080,7 +7080,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.01920141698792577</v>
+        <v>0.01950645894976333</v>
       </c>
       <c r="C2" t="n">
         <v>15.05740487737325</v>
@@ -7194,7 +7194,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02192566700978205</v>
+        <v>0.022541958023794</v>
       </c>
       <c r="C2" t="n">
         <v>22.93071727096042</v>
@@ -7308,7 +7308,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.0207838750211522</v>
+        <v>0.0209500000346452</v>
       </c>
       <c r="C2" t="n">
         <v>17.71264276554266</v>
@@ -7422,7 +7422,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02363608300220221</v>
+        <v>0.02280104201054201</v>
       </c>
       <c r="C2" t="n">
         <v>17.21129367079983</v>
@@ -7536,7 +7536,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02214041701517999</v>
+        <v>0.02121824998175725</v>
       </c>
       <c r="C2" t="n">
         <v>20.80983841346563</v>
@@ -7650,7 +7650,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02520279202144593</v>
+        <v>0.02369237499078736</v>
       </c>
       <c r="C2" t="n">
         <v>17.45391221435329</v>
@@ -7764,7 +7764,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02308645902667195</v>
+        <v>0.02225304098101333</v>
       </c>
       <c r="C2" t="n">
         <v>19.35257674063202</v>
@@ -7878,7 +7878,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02163783396827057</v>
+        <v>0.0207660419982858</v>
       </c>
       <c r="C2" t="n">
         <v>22.35189399632039</v>
@@ -7992,7 +7992,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02069391700206324</v>
+        <v>0.0204757500323467</v>
       </c>
       <c r="C2" t="n">
         <v>18.01859019881032</v>
@@ -8106,7 +8106,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.01783550000982359</v>
+        <v>0.01754233299288899</v>
       </c>
       <c r="C2" t="n">
         <v>22.12890953330058</v>
@@ -8220,7 +8220,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.01782000000821427</v>
+        <v>0.01727716595632955</v>
       </c>
       <c r="C2" t="n">
         <v>19.13023140604607</v>
@@ -8334,7 +8334,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02389599999878556</v>
+        <v>0.02715641696704552</v>
       </c>
       <c r="C2" t="n">
         <v>14.32201607185219</v>
@@ -8448,7 +8448,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02301162498770282</v>
+        <v>0.02248120802687481</v>
       </c>
       <c r="C2" t="n">
         <v>23.1684976854833</v>
@@ -8562,7 +8562,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02160929096862674</v>
+        <v>0.02020337496651337</v>
       </c>
       <c r="C2" t="n">
         <v>18.72448189562278</v>
@@ -8676,7 +8676,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02238254103576764</v>
+        <v>0.02122812496963888</v>
       </c>
       <c r="C2" t="n">
         <v>16.06950484980027</v>
@@ -8790,7 +8790,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02262879197951406</v>
+        <v>0.02224075002595782</v>
       </c>
       <c r="C2" t="n">
         <v>15.18635083795624</v>
@@ -8904,7 +8904,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.01792274997569621</v>
+        <v>0.01761875004740432</v>
       </c>
       <c r="C2" t="n">
         <v>14.74680990044796</v>
@@ -9018,7 +9018,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.01948766701389104</v>
+        <v>0.01915200002258644</v>
       </c>
       <c r="C2" t="n">
         <v>20.18600795826394</v>
@@ -9132,7 +9132,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.0230927910306491</v>
+        <v>0.02327070897445083</v>
       </c>
       <c r="C2" t="n">
         <v>13.72188318471989</v>
@@ -9246,7 +9246,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02011241699801758</v>
+        <v>0.01949195901397616</v>
       </c>
       <c r="C2" t="n">
         <v>20.62117239421754</v>
@@ -9360,7 +9360,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02072425000369549</v>
+        <v>0.02060108399018645</v>
       </c>
       <c r="C2" t="n">
         <v>15.68624644771859</v>
@@ -9474,7 +9474,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02383183303754777</v>
+        <v>0.02375858399318531</v>
       </c>
       <c r="C2" t="n">
         <v>16.45028071224679</v>
@@ -9588,7 +9588,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02577712503261864</v>
+        <v>0.02537591703003272</v>
       </c>
       <c r="C2" t="n">
         <v>24.63502149030433</v>
@@ -9702,7 +9702,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.01987350004492328</v>
+        <v>0.01919525000266731</v>
       </c>
       <c r="C2" t="n">
         <v>21.93135520138235</v>
@@ -9816,7 +9816,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02084308303892612</v>
+        <v>0.0201390830334276</v>
       </c>
       <c r="C2" t="n">
         <v>17.70385262850725</v>
@@ -9930,7 +9930,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02330608404008672</v>
+        <v>0.02321700000902638</v>
       </c>
       <c r="C2" t="n">
         <v>15.57655990615665</v>
@@ -10044,7 +10044,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02708154200809076</v>
+        <v>0.02674670802662149</v>
       </c>
       <c r="C2" t="n">
         <v>20.89749717041111</v>
@@ -10158,7 +10158,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02207716699922457</v>
+        <v>0.02158229099586606</v>
       </c>
       <c r="C2" t="n">
         <v>16.1677780976814</v>
@@ -10272,7 +10272,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02187208301620558</v>
+        <v>0.02184595802100375</v>
       </c>
       <c r="C2" t="n">
         <v>15.62835064422036</v>
@@ -10386,7 +10386,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.01924824999878183</v>
+        <v>0.01886820903746411</v>
       </c>
       <c r="C2" t="n">
         <v>16.81806735896556</v>
@@ -10500,7 +10500,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.0210511659970507</v>
+        <v>0.02104237501043826</v>
       </c>
       <c r="C2" t="n">
         <v>18.78315794836075</v>
@@ -10614,7 +10614,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02761712501524016</v>
+        <v>0.02783216704847291</v>
       </c>
       <c r="C2" t="n">
         <v>15.31219211528135</v>
@@ -10728,7 +10728,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02454629103885964</v>
+        <v>0.02464762498857453</v>
       </c>
       <c r="C2" t="n">
         <v>19.29246871496888</v>
@@ -10842,7 +10842,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.01717033400200307</v>
+        <v>0.01706112502142787</v>
       </c>
       <c r="C2" t="n">
         <v>19.02461826969006</v>
@@ -10956,7 +10956,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02321916696382686</v>
+        <v>0.02221516601275653</v>
       </c>
       <c r="C2" t="n">
         <v>17.95044638345265</v>
@@ -11070,7 +11070,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02176604204578325</v>
+        <v>0.02103362500201911</v>
       </c>
       <c r="C2" t="n">
         <v>15.82297057283138</v>
@@ -11184,7 +11184,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.0201610840158537</v>
+        <v>0.01948462502332404</v>
       </c>
       <c r="C2" t="n">
         <v>17.45872264627423</v>
@@ -11298,7 +11298,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.01815995801007375</v>
+        <v>0.01756116701290011</v>
       </c>
       <c r="C2" t="n">
         <v>16.76390499318886</v>
@@ -11412,7 +11412,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.01874537504045293</v>
+        <v>0.01786770904436707</v>
       </c>
       <c r="C2" t="n">
         <v>18.89858989195232</v>
@@ -11526,7 +11526,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02785629098070785</v>
+        <v>0.02686962502775714</v>
       </c>
       <c r="C2" t="n">
         <v>23.32658524368457</v>
@@ -11640,7 +11640,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.025851208018139</v>
+        <v>0.02417845802847296</v>
       </c>
       <c r="C2" t="n">
         <v>14.99431487412712</v>
@@ -11754,7 +11754,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02232058299705386</v>
+        <v>0.02144162502372637</v>
       </c>
       <c r="C2" t="n">
         <v>19.02935228003166</v>
@@ -11868,7 +11868,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.02167058299528435</v>
+        <v>0.02020958397770301</v>
       </c>
       <c r="C2" t="n">
         <v>25.10324692851615</v>

</xml_diff>